<commit_message>
Files Renamed changes Nov 18 2023
</commit_message>
<xml_diff>
--- a/TestData/T2286_T2287_TMTC0001544_TMTC0001548_VerifyRateGenerationToStaffWithDifferentTitleInSummaryAndDetailsLogTab.xlsx
+++ b/TestData/T2286_T2287_TMTC0001544_TMTC0001548_VerifyRateGenerationToStaffWithDifferentTitleInSummaryAndDetailsLogTab.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20390"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26924"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SMittal0207\source\repos\SalesForce_Project\TestData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB632BF2-2D6A-41B2-84E9-3D43AFEA6040}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B043745-9B0C-4500-A17A-FB6D71299CFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="12756" windowHeight="2976" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="5" r:id="rId1"/>
@@ -144,10 +144,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -431,7 +432,7 @@
   <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.44140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18.5546875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -552,15 +553,15 @@
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="30.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="31.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>8</v>
       </c>
     </row>
@@ -582,18 +583,18 @@
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="30.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="26.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>13</v>
       </c>
     </row>

</xml_diff>